<commit_message>
Plan final: Valle 101,2 h, Risaralda con reparto nuevo, anillos segun la Circular 73 y daño declarado sin verdes falsos
Valle, 90 sedes: 101,23 h con todas las coordenadas revisadas. Risaralda: 45,39 h
y 37 dias con el reparto que encontro el solucionador (Apia al grupo del norte,
Santa Rosa de Cabal al de Pereira).

Anillo verde solo para las 3 sedes con concepto «Habitable» aprobado por la mesa:
la Circular 73 de la UNGRD manda los colegios directo a la evaluacion detallada,
asi que la afectacion menor declarada no saca a nadie de la visita. Anillo blanco:
sin concepto tecnico ni reporte del rector. La ficha y el globo dicen «Reporte
rector al MEN» y «Reporte FFIE 2026».

Pestaña del pedido del MEN: en la capa «sin afectacion» es lo que queda cuando la
sede no reporto; esas 223 pasan de verde a gris («No reporto al MEN»). A 14 de
Dosquebradas que reportaron daño con el nivel vacio se les toma el nivel del
estado declarado.
</commit_message>
<xml_diff>
--- a/public/datos/plan_cuadrillas_por_municipio.xlsx
+++ b/public/datos/plan_cuadrillas_por_municipio.xlsx
@@ -3090,7 +3090,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>camino rural sin categoria</t>
+          <t>camino destapado</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
@@ -3100,12 +3100,12 @@
       </c>
       <c r="Z20" t="inlineStr">
         <is>
-          <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 0 m de esa vía.</t>
+          <t>OpenStreetMap la marca como «track», la clase de los caminos de uso agrícola o forestal. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 4 m de esa vía.</t>
         </is>
       </c>
       <c r="AA20" t="inlineStr">
         <is>
-          <t>Calle 8</t>
+          <t>Calle 7B</t>
         </is>
       </c>
       <c r="AB20" t="inlineStr">
@@ -3214,22 +3214,17 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>camino rural sin categoria</t>
+          <t>calle de casco urbano</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>difícil</t>
+          <t>fácil</t>
         </is>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
-          <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 17 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AA21" t="inlineStr">
-        <is>
-          <t>Calle 7</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «service»). La sede queda a 3 m de esa vía.</t>
         </is>
       </c>
       <c r="AB21" t="inlineStr">
@@ -3279,11 +3274,6 @@
           <t>LA MILAGROSA</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>INSTITUCION EDUCATIVA LA MILAGROSA</t>
-        </is>
-      </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
           <t>176520002279</t>
@@ -3292,16 +3282,6 @@
       <c r="K22" t="inlineStr">
         <is>
           <t>Palmira</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>CR 28 NO 33 12</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -3325,36 +3305,6 @@
       </c>
       <c r="S22" t="n">
         <v>0.8</v>
-      </c>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>Afectación menor</t>
-        </is>
-      </c>
-      <c r="W22" t="inlineStr">
-        <is>
-          <t>Bajo</t>
-        </is>
-      </c>
-      <c r="X22" t="inlineStr">
-        <is>
-          <t>calle de casco urbano</t>
-        </is>
-      </c>
-      <c r="Y22" t="inlineStr">
-        <is>
-          <t>fácil</t>
-        </is>
-      </c>
-      <c r="Z22" t="inlineStr">
-        <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 21 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AA22" t="inlineStr">
-        <is>
-          <t>Calle 34</t>
-        </is>
       </c>
       <c r="AB22" t="inlineStr">
         <is>
@@ -3403,11 +3353,6 @@
           <t>TULIO RAFFO</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>INSTITUCION EDUCATIVA JORGE ELIECER GAITAN</t>
-        </is>
-      </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
           <t>176520001949</t>
@@ -3416,16 +3361,6 @@
       <c r="K23" t="inlineStr">
         <is>
           <t>Palmira</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>CLL 37 NO 42A 110</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -3449,36 +3384,6 @@
       </c>
       <c r="S23" t="n">
         <v>4.8</v>
-      </c>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W23" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="X23" t="inlineStr">
-        <is>
-          <t>calle de casco urbano</t>
-        </is>
-      </c>
-      <c r="Y23" t="inlineStr">
-        <is>
-          <t>fácil</t>
-        </is>
-      </c>
-      <c r="Z23" t="inlineStr">
-        <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 20 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AA23" t="inlineStr">
-        <is>
-          <t>Calle 38</t>
-        </is>
       </c>
       <c r="AB23" t="inlineStr">
         <is>
@@ -3527,11 +3432,6 @@
           <t>GREGORIO HERNANDEZ</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>INSTITUCION EDUCATIVA LA MILAGROSA</t>
-        </is>
-      </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
           <t>176520001825</t>
@@ -3540,16 +3440,6 @@
       <c r="K24" t="inlineStr">
         <is>
           <t>Palmira</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>CLL 34 NO 31 71</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -3573,36 +3463,6 @@
       </c>
       <c r="S24" t="n">
         <v>4.8</v>
-      </c>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W24" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="X24" t="inlineStr">
-        <is>
-          <t>calle de casco urbano</t>
-        </is>
-      </c>
-      <c r="Y24" t="inlineStr">
-        <is>
-          <t>fácil</t>
-        </is>
-      </c>
-      <c r="Z24" t="inlineStr">
-        <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 8 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AA24" t="inlineStr">
-        <is>
-          <t>Calle 34</t>
-        </is>
       </c>
       <c r="AB24" t="inlineStr">
         <is>
@@ -3651,11 +3511,6 @@
           <t>ALFONSO CABAL MADRIÑAN</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>INSTITUCION EDUCATIVA MERCEDES ABREGO</t>
-        </is>
-      </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
           <t>176520001761</t>
@@ -3664,16 +3519,6 @@
       <c r="K25" t="inlineStr">
         <is>
           <t>Palmira</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>CL 40 KR 12 ESQ</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -3697,36 +3542,6 @@
       </c>
       <c r="S25" t="n">
         <v>4</v>
-      </c>
-      <c r="V25" t="inlineStr">
-        <is>
-          <t>Afectación parcial</t>
-        </is>
-      </c>
-      <c r="W25" t="inlineStr">
-        <is>
-          <t>Moderado</t>
-        </is>
-      </c>
-      <c r="X25" t="inlineStr">
-        <is>
-          <t>calle de casco urbano</t>
-        </is>
-      </c>
-      <c r="Y25" t="inlineStr">
-        <is>
-          <t>fácil</t>
-        </is>
-      </c>
-      <c r="Z25" t="inlineStr">
-        <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 12 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AA25" t="inlineStr">
-        <is>
-          <t>Calle 40</t>
-        </is>
       </c>
       <c r="AB25" t="inlineStr">
         <is>
@@ -3775,11 +3590,6 @@
           <t>JOSE MARIA CORDOBA</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>INSTITUCION EDUCATIVA LA MILAGROSA</t>
-        </is>
-      </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
           <t>176520001736</t>
@@ -3788,16 +3598,6 @@
       <c r="K26" t="inlineStr">
         <is>
           <t>Palmira</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>CR 22 CLL  33 ESQ</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -3821,36 +3621,6 @@
       </c>
       <c r="S26" t="n">
         <v>4</v>
-      </c>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>Afectación menor</t>
-        </is>
-      </c>
-      <c r="W26" t="inlineStr">
-        <is>
-          <t>Bajo</t>
-        </is>
-      </c>
-      <c r="X26" t="inlineStr">
-        <is>
-          <t>calle de casco urbano</t>
-        </is>
-      </c>
-      <c r="Y26" t="inlineStr">
-        <is>
-          <t>fácil</t>
-        </is>
-      </c>
-      <c r="Z26" t="inlineStr">
-        <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 12 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AA26" t="inlineStr">
-        <is>
-          <t>Calle 33</t>
-        </is>
       </c>
       <c r="AB26" t="inlineStr">
         <is>
@@ -4023,11 +3793,6 @@
           <t>SANTA TERESITA (U)</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>INSTITUCION EDUCATIVA DOMINGO IRURITA</t>
-        </is>
-      </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
           <t>176520001990</t>
@@ -4036,16 +3801,6 @@
       <c r="K28" t="inlineStr">
         <is>
           <t>Palmira</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>KR 24 A 20 97</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -4069,31 +3824,6 @@
       </c>
       <c r="S28" t="n">
         <v>3.2</v>
-      </c>
-      <c r="V28" t="inlineStr">
-        <is>
-          <t>Afectación parcial</t>
-        </is>
-      </c>
-      <c r="W28" t="inlineStr">
-        <is>
-          <t>Moderado</t>
-        </is>
-      </c>
-      <c r="X28" t="inlineStr">
-        <is>
-          <t>calle de casco urbano</t>
-        </is>
-      </c>
-      <c r="Y28" t="inlineStr">
-        <is>
-          <t>fácil</t>
-        </is>
-      </c>
-      <c r="Z28" t="inlineStr">
-        <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 27 m de esa vía.</t>
-        </is>
       </c>
       <c r="AB28" t="inlineStr">
         <is>
@@ -4261,11 +3991,6 @@
           <t>SANTISIMA TRINIDAD</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>INSTITUCION EDUCATIVA ALFONSO LOPEZ PUMAREJO</t>
-        </is>
-      </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
           <t>176520002317</t>
@@ -4274,16 +3999,6 @@
       <c r="K30" t="inlineStr">
         <is>
           <t>Palmira</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>CLL 31NO 15 44</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -4307,31 +4022,6 @@
       </c>
       <c r="S30" t="n">
         <v>4</v>
-      </c>
-      <c r="V30" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W30" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="X30" t="inlineStr">
-        <is>
-          <t>calle de casco urbano</t>
-        </is>
-      </c>
-      <c r="Y30" t="inlineStr">
-        <is>
-          <t>fácil</t>
-        </is>
-      </c>
-      <c r="Z30" t="inlineStr">
-        <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «service»). La sede queda a 41 m de esa vía.</t>
-        </is>
       </c>
       <c r="AB30" t="inlineStr">
         <is>
@@ -4380,11 +4070,6 @@
           <t>PRAXEDES ESPINOSA</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>INSTITUCION EDUCATIVA ALFONSO LOPEZ PUMAREJO</t>
-        </is>
-      </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
           <t>176520002201</t>
@@ -4393,16 +4078,6 @@
       <c r="K31" t="inlineStr">
         <is>
           <t>Palmira</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>CLL 2ENO 31 20</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -4426,36 +4101,6 @@
       </c>
       <c r="S31" t="n">
         <v>4.8</v>
-      </c>
-      <c r="V31" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W31" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="X31" t="inlineStr">
-        <is>
-          <t>calle de casco urbano</t>
-        </is>
-      </c>
-      <c r="Y31" t="inlineStr">
-        <is>
-          <t>fácil</t>
-        </is>
-      </c>
-      <c r="Z31" t="inlineStr">
-        <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 17 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AA31" t="inlineStr">
-        <is>
-          <t>Calle 32A</t>
-        </is>
       </c>
       <c r="AB31" t="inlineStr">
         <is>
@@ -4504,11 +4149,6 @@
           <t>AGUSTIN CODAZZI</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>INSTITUCION EDUCATIVA ALFONSO LOPEZ PUMAREJO</t>
-        </is>
-      </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
           <t>176520001795</t>
@@ -4517,16 +4157,6 @@
       <c r="K32" t="inlineStr">
         <is>
           <t>Palmira</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>CLL 30 NO 7  40</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -4550,36 +4180,6 @@
       </c>
       <c r="S32" t="n">
         <v>4.8</v>
-      </c>
-      <c r="V32" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W32" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="X32" t="inlineStr">
-        <is>
-          <t>calle de casco urbano</t>
-        </is>
-      </c>
-      <c r="Y32" t="inlineStr">
-        <is>
-          <t>fácil</t>
-        </is>
-      </c>
-      <c r="Z32" t="inlineStr">
-        <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 15 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AA32" t="inlineStr">
-        <is>
-          <t>Calle 30</t>
-        </is>
       </c>
       <c r="AB32" t="inlineStr">
         <is>
@@ -4628,11 +4228,6 @@
           <t>MARIA ANTONIA PENAGOS</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>INSTITUCION EDUCATIVA MARIA ANTONIA PENAGOS</t>
-        </is>
-      </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
           <t>176520002520</t>
@@ -4641,16 +4236,6 @@
       <c r="K33" t="inlineStr">
         <is>
           <t>Palmira</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>KR 31 15 A 40</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -4674,36 +4259,6 @@
       </c>
       <c r="S33" t="n">
         <v>4.5</v>
-      </c>
-      <c r="V33" t="inlineStr">
-        <is>
-          <t>Afectación menor</t>
-        </is>
-      </c>
-      <c r="W33" t="inlineStr">
-        <is>
-          <t>Bajo</t>
-        </is>
-      </c>
-      <c r="X33" t="inlineStr">
-        <is>
-          <t>calle de casco urbano</t>
-        </is>
-      </c>
-      <c r="Y33" t="inlineStr">
-        <is>
-          <t>fácil</t>
-        </is>
-      </c>
-      <c r="Z33" t="inlineStr">
-        <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 14 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AA33" t="inlineStr">
-        <is>
-          <t>Carrera 30</t>
-        </is>
       </c>
       <c r="AB33" t="inlineStr">
         <is>
@@ -4752,11 +4307,6 @@
           <t>FRANCISCO DE PAULA SANTANDER</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>INSTITUCION EDUCATIVA MARIA ANTONIA PENAGOS</t>
-        </is>
-      </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
           <t>176520001817</t>
@@ -4765,16 +4315,6 @@
       <c r="K34" t="inlineStr">
         <is>
           <t>Palmira</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>CR 27 NO  25 50</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -4798,36 +4338,6 @@
       </c>
       <c r="S34" t="n">
         <v>4.5</v>
-      </c>
-      <c r="V34" t="inlineStr">
-        <is>
-          <t>Afectación menor</t>
-        </is>
-      </c>
-      <c r="W34" t="inlineStr">
-        <is>
-          <t>Bajo</t>
-        </is>
-      </c>
-      <c r="X34" t="inlineStr">
-        <is>
-          <t>calle de casco urbano</t>
-        </is>
-      </c>
-      <c r="Y34" t="inlineStr">
-        <is>
-          <t>fácil</t>
-        </is>
-      </c>
-      <c r="Z34" t="inlineStr">
-        <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 8 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AA34" t="inlineStr">
-        <is>
-          <t>Carrera 27</t>
-        </is>
       </c>
       <c r="AB34" t="inlineStr">
         <is>
@@ -4876,11 +4386,6 @@
           <t>MONSEÑOR GUILLERMO BECERRA</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>INSTITUCION EDUCATIVA DOMINGO IRURITA</t>
-        </is>
-      </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
           <t>176520001884</t>
@@ -4889,16 +4394,6 @@
       <c r="K35" t="inlineStr">
         <is>
           <t>Palmira</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>CR 35 NO 25B 10</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -4922,36 +4417,6 @@
       </c>
       <c r="S35" t="n">
         <v>4.7</v>
-      </c>
-      <c r="V35" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W35" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="X35" t="inlineStr">
-        <is>
-          <t>calle de casco urbano</t>
-        </is>
-      </c>
-      <c r="Y35" t="inlineStr">
-        <is>
-          <t>fácil</t>
-        </is>
-      </c>
-      <c r="Z35" t="inlineStr">
-        <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 31 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AA35" t="inlineStr">
-        <is>
-          <t>Carrera 35</t>
-        </is>
       </c>
       <c r="AB35" t="inlineStr">
         <is>
@@ -5059,22 +4524,22 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>camino rural sin categoria</t>
+          <t>via terciaria</t>
         </is>
       </c>
       <c r="Y36" t="inlineStr">
         <is>
-          <t>difícil</t>
+          <t>fácil</t>
         </is>
       </c>
       <c r="Z36" t="inlineStr">
         <is>
-          <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 16 m de esa vía.</t>
+          <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 35 m de esa vía.</t>
         </is>
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>Calle 23</t>
+          <t>Carrera 33A</t>
         </is>
       </c>
       <c r="AB36" t="inlineStr">
@@ -5124,11 +4589,6 @@
           <t>VASCO NUÑEZ DE BALBOA</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>INSTITUCION EDUCATIVA SEMILLA DE LA ESPERANZA</t>
-        </is>
-      </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
           <t>276520000823</t>
@@ -5137,16 +4597,6 @@
       <c r="K37" t="inlineStr">
         <is>
           <t>Palmira</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>CORREG AMAIME</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -5170,31 +4620,6 @@
       </c>
       <c r="S37" t="n">
         <v>22.4</v>
-      </c>
-      <c r="V37" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W37" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="X37" t="inlineStr">
-        <is>
-          <t>calle de casco urbano</t>
-        </is>
-      </c>
-      <c r="Y37" t="inlineStr">
-        <is>
-          <t>fácil</t>
-        </is>
-      </c>
-      <c r="Z37" t="inlineStr">
-        <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «service»). La sede queda a 58 m de esa vía.</t>
-        </is>
       </c>
       <c r="AB37" t="inlineStr">
         <is>
@@ -5243,11 +4668,6 @@
           <t>BOSQUES DEL EDEN</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>INSTITUCION EDUCATIVA ANTONIO LIZARAZO</t>
-        </is>
-      </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
           <t>176520800167</t>
@@ -5256,16 +4676,6 @@
       <c r="K38" t="inlineStr">
         <is>
           <t>Palmira</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>IND KR 35 CL 60 EQ</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -5289,36 +4699,6 @@
       </c>
       <c r="S38" t="n">
         <v>22.4</v>
-      </c>
-      <c r="V38" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W38" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="X38" t="inlineStr">
-        <is>
-          <t>via terciaria</t>
-        </is>
-      </c>
-      <c r="Y38" t="inlineStr">
-        <is>
-          <t>fácil</t>
-        </is>
-      </c>
-      <c r="Z38" t="inlineStr">
-        <is>
-          <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 8 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AA38" t="inlineStr">
-        <is>
-          <t>Carrera 35</t>
-        </is>
       </c>
       <c r="AB38" t="inlineStr">
         <is>
@@ -5367,11 +4747,6 @@
           <t>HELIODORO VILLEGAS</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>INSTITUCION EDUCATIVA SEMILLA DE LA ESPERANZA</t>
-        </is>
-      </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
           <t>276520002010</t>
@@ -5380,16 +4755,6 @@
       <c r="K39" t="inlineStr">
         <is>
           <t>Palmira</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>VDA LA PAMPA</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -5413,31 +4778,6 @@
       </c>
       <c r="S39" t="n">
         <v>23.1</v>
-      </c>
-      <c r="V39" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W39" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="X39" t="inlineStr">
-        <is>
-          <t>camino rural sin categoria</t>
-        </is>
-      </c>
-      <c r="Y39" t="inlineStr">
-        <is>
-          <t>difícil</t>
-        </is>
-      </c>
-      <c r="Z39" t="inlineStr">
-        <is>
-          <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 60 m de esa vía.</t>
-        </is>
       </c>
       <c r="AB39" t="inlineStr">
         <is>
@@ -5486,11 +4826,6 @@
           <t>SEMILLA DE LA ESPERANZA</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>INSTITUCION EDUCATIVA SEMILLA DE LA ESPERANZA</t>
-        </is>
-      </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
           <t>276520005248</t>
@@ -5499,16 +4834,6 @@
       <c r="K40" t="inlineStr">
         <is>
           <t>Palmira</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>CORREG AMAIME</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -5532,31 +4857,6 @@
       </c>
       <c r="S40" t="n">
         <v>23.1</v>
-      </c>
-      <c r="V40" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W40" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="X40" t="inlineStr">
-        <is>
-          <t>via principal pavimentada</t>
-        </is>
-      </c>
-      <c r="Y40" t="inlineStr">
-        <is>
-          <t>fácil</t>
-        </is>
-      </c>
-      <c r="Z40" t="inlineStr">
-        <is>
-          <t>La vía de entrada es via principal pavimentada según OpenStreetMap (clase «secondary»). La sede queda a 134 m de esa vía.</t>
-        </is>
       </c>
       <c r="AB40" t="inlineStr">
         <is>
@@ -5605,11 +4905,6 @@
           <t>SUSANA LOPEZ DE VALENCIA</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>INSTITUCION EDUCATIVA MARIA ANTONIA PENAGOS</t>
-        </is>
-      </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
           <t>176520002694</t>
@@ -5618,16 +4913,6 @@
       <c r="K41" t="inlineStr">
         <is>
           <t>Palmira</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>KR 26 CL 12 ESQ</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -5651,36 +4936,6 @@
       </c>
       <c r="S41" t="n">
         <v>17.8</v>
-      </c>
-      <c r="V41" t="inlineStr">
-        <is>
-          <t>Afectación menor</t>
-        </is>
-      </c>
-      <c r="W41" t="inlineStr">
-        <is>
-          <t>Bajo</t>
-        </is>
-      </c>
-      <c r="X41" t="inlineStr">
-        <is>
-          <t>calle de casco urbano</t>
-        </is>
-      </c>
-      <c r="Y41" t="inlineStr">
-        <is>
-          <t>fácil</t>
-        </is>
-      </c>
-      <c r="Z41" t="inlineStr">
-        <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 20 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AA41" t="inlineStr">
-        <is>
-          <t>Calle 12</t>
-        </is>
       </c>
       <c r="AB41" t="inlineStr">
         <is>
@@ -5729,11 +4984,6 @@
           <t>MEGACOLEGIO DEL SUR</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>INSTITUCION EDUCATIVA MARIA ANTONIA PENAGOS</t>
-        </is>
-      </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
           <t>176520800222</t>
@@ -5742,16 +4992,6 @@
       <c r="K42" t="inlineStr">
         <is>
           <t>PALMIRA</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">IND CL 5 29 107 </t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -5775,36 +5015,6 @@
       </c>
       <c r="S42" t="n">
         <v>17.8</v>
-      </c>
-      <c r="V42" t="inlineStr">
-        <is>
-          <t>Afectación menor</t>
-        </is>
-      </c>
-      <c r="W42" t="inlineStr">
-        <is>
-          <t>Bajo</t>
-        </is>
-      </c>
-      <c r="X42" t="inlineStr">
-        <is>
-          <t>calle de casco urbano</t>
-        </is>
-      </c>
-      <c r="Y42" t="inlineStr">
-        <is>
-          <t>fácil</t>
-        </is>
-      </c>
-      <c r="Z42" t="inlineStr">
-        <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 33 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AA42" t="inlineStr">
-        <is>
-          <t>Calle 5</t>
-        </is>
       </c>
       <c r="AB42" t="inlineStr">
         <is>
@@ -7845,7 +7055,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>Tulua</t>
+          <t>Andalucia</t>
         </is>
       </c>
       <c r="P58" t="n">
@@ -7855,10 +7065,10 @@
         <v>13.08</v>
       </c>
       <c r="R58" t="n">
-        <v>104.5</v>
+        <v>92.3</v>
       </c>
       <c r="S58" t="n">
-        <v>90.09999999999999</v>
+        <v>77.8</v>
       </c>
       <c r="T58" t="inlineStr">
         <is>
@@ -7979,20 +7189,20 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>Tulua</t>
+          <t>Andalucia</t>
         </is>
       </c>
       <c r="P59" t="n">
         <v>13.08</v>
       </c>
       <c r="Q59" t="n">
-        <v>55.52</v>
+        <v>43.36</v>
       </c>
       <c r="R59" t="n">
-        <v>104.5</v>
+        <v>92.3</v>
       </c>
       <c r="S59" t="n">
-        <v>90.09999999999999</v>
+        <v>77.8</v>
       </c>
       <c r="T59" t="inlineStr">
         <is>
@@ -8073,74 +7283,84 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Tuluá</t>
+          <t>BID (43)</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>SEDE PRINCIPAL LICEO MODERNO</t>
+          <t>SAN ISIDRO</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA MODERNA DE TULUA</t>
+          <t>INSTITUCION EDUCATIVA SAN ISIDRO</t>
         </is>
       </c>
       <c r="J60" s="3" t="inlineStr">
         <is>
-          <t>176834000106</t>
+          <t>276828000174</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>Tuluá</t>
+          <t>TRUJILLO</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>Urbana</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>IND CALLE 27 NO. 6AW 240</t>
+          <t>CORREGIMIENTO EL TABOR PUENTE BLANCO</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
         <is>
+          <t>Andalucia</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
           <t>Tulua</t>
         </is>
       </c>
-      <c r="O60" t="inlineStr">
-        <is>
-          <t>Tulua</t>
-        </is>
-      </c>
       <c r="P60" t="n">
-        <v>7.41</v>
+        <v>90.59</v>
       </c>
       <c r="Q60" t="n">
-        <v>42.09</v>
+        <v>69.08</v>
       </c>
       <c r="R60" t="n">
-        <v>100.2</v>
+        <v>159.7</v>
       </c>
       <c r="S60" t="n">
-        <v>57</v>
+        <v>86.3</v>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>Habitable</t>
+        </is>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>aprobado por la mesa</t>
+        </is>
       </c>
       <c r="V60" t="inlineStr">
         <is>
-          <t>Colapso parcial</t>
+          <t>Afectación parcial</t>
         </is>
       </c>
       <c r="W60" t="inlineStr">
         <is>
-          <t>Critico</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="X60" t="inlineStr">
         <is>
-          <t>via principal pavimentada</t>
+          <t>via terciaria</t>
         </is>
       </c>
       <c r="Y60" t="inlineStr">
@@ -8150,12 +7370,12 @@
       </c>
       <c r="Z60" t="inlineStr">
         <is>
-          <t>La vía de entrada es via principal pavimentada según OpenStreetMap (clase «secondary»). La sede queda a 12 m de esa vía.</t>
+          <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 33 m de esa vía.</t>
         </is>
       </c>
       <c r="AA60" t="inlineStr">
         <is>
-          <t>Calle 27</t>
+          <t>TRUJILLO - LA SONORA CRUCE VIA 23VL13-1 K64+160</t>
         </is>
       </c>
       <c r="AB60" t="inlineStr">
@@ -8164,10 +7384,10 @@
         </is>
       </c>
       <c r="AC60" t="n">
-        <v>4.088515899</v>
+        <v>4.210564</v>
       </c>
       <c r="AD60" t="n">
-        <v>-76.22009</v>
+        <v>-76.38158300000001</v>
       </c>
     </row>
     <row r="61">
@@ -8186,48 +7406,48 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>miércoles</t>
+          <t>jueves</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>BID (43)</t>
+          <t>Tuluá</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>JOSE MARIA CORDOBA</t>
+          <t>SEDE PRINCIPAL LICEO MODERNO</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA HERNANDO LLORENTE ARROYO</t>
+          <t>INSTITUCION EDUCATIVA MODERNA DE TULUA</t>
         </is>
       </c>
       <c r="J61" s="3" t="inlineStr">
         <is>
-          <t>276616000212</t>
+          <t>176834000106</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>RIOFRIO</t>
+          <t>Tuluá</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>CORREG SALONICA</t>
+          <t>IND CALLE 27 NO. 6AW 240</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -8241,10 +7461,10 @@
         </is>
       </c>
       <c r="P61" t="n">
+        <v>7.41</v>
+      </c>
+      <c r="Q61" t="n">
         <v>42.09</v>
-      </c>
-      <c r="Q61" t="n">
-        <v>50.65</v>
       </c>
       <c r="R61" t="n">
         <v>100.2</v>
@@ -8252,19 +7472,9 @@
       <c r="S61" t="n">
         <v>57</v>
       </c>
-      <c r="T61" t="inlineStr">
-        <is>
-          <t>Peligro de colapso</t>
-        </is>
-      </c>
-      <c r="U61" t="inlineStr">
-        <is>
-          <t>en revisión de la mesa</t>
-        </is>
-      </c>
       <c r="V61" t="inlineStr">
         <is>
-          <t>Riesgo inminente de colapso</t>
+          <t>Colapso parcial</t>
         </is>
       </c>
       <c r="W61" t="inlineStr">
@@ -8274,7 +7484,7 @@
       </c>
       <c r="X61" t="inlineStr">
         <is>
-          <t>calle de casco urbano</t>
+          <t>via principal pavimentada</t>
         </is>
       </c>
       <c r="Y61" t="inlineStr">
@@ -8284,12 +7494,12 @@
       </c>
       <c r="Z61" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 26 m de esa vía.</t>
+          <t>La vía de entrada es via principal pavimentada según OpenStreetMap (clase «secondary»). La sede queda a 12 m de esa vía.</t>
         </is>
       </c>
       <c r="AA61" t="inlineStr">
         <is>
-          <t>SALONICA CRUCE CON VIA 23VL13-1 EN K44+300</t>
+          <t>Calle 27</t>
         </is>
       </c>
       <c r="AB61" t="inlineStr">
@@ -8298,10 +7508,10 @@
         </is>
       </c>
       <c r="AC61" t="n">
-        <v>4.1258314</v>
+        <v>4.088515899</v>
       </c>
       <c r="AD61" t="n">
-        <v>-76.3722336</v>
+        <v>-76.22009</v>
       </c>
     </row>
     <row r="62">
@@ -8327,41 +7537,41 @@
         <v>10</v>
       </c>
       <c r="F62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Tuluá</t>
+          <t>BID (43)</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>SEDE INSTITUTO CAMPESTRE SANTA CECILIA</t>
+          <t>JOSE MARIA CORDOBA</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA MODERNA DE TULUA</t>
+          <t>INSTITUCION EDUCATIVA HERNANDO LLORENTE ARROYO</t>
         </is>
       </c>
       <c r="J62" s="3" t="inlineStr">
         <is>
-          <t>176834000599</t>
+          <t>276616000212</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>Tuluá</t>
+          <t>RIOFRIO</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>Urbana</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>IND CALLE 27 NO 6AW 240</t>
+          <t>CORREG SALONICA</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -8375,40 +7585,55 @@
         </is>
       </c>
       <c r="P62" t="n">
-        <v>9.890000000000001</v>
+        <v>42.09</v>
       </c>
       <c r="Q62" t="n">
-        <v>32.44</v>
+        <v>50.65</v>
       </c>
       <c r="R62" t="n">
-        <v>84.09999999999999</v>
+        <v>100.2</v>
       </c>
       <c r="S62" t="n">
-        <v>59</v>
+        <v>57</v>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>Peligro de colapso</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>en revisión de la mesa</t>
+        </is>
       </c>
       <c r="V62" t="inlineStr">
         <is>
-          <t>Afectación parcial</t>
+          <t>Riesgo inminente de colapso</t>
         </is>
       </c>
       <c r="W62" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Critico</t>
         </is>
       </c>
       <c r="X62" t="inlineStr">
         <is>
-          <t>camino destapado</t>
+          <t>calle de casco urbano</t>
         </is>
       </c>
       <c r="Y62" t="inlineStr">
         <is>
-          <t>difícil</t>
+          <t>fácil</t>
         </is>
       </c>
       <c r="Z62" t="inlineStr">
         <is>
-          <t>OpenStreetMap la marca como «track», la clase de los caminos de uso agrícola o forestal. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 50 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 26 m de esa vía.</t>
+        </is>
+      </c>
+      <c r="AA62" t="inlineStr">
+        <is>
+          <t>SALONICA CRUCE CON VIA 23VL13-1 EN K44+300</t>
         </is>
       </c>
       <c r="AB62" t="inlineStr">
@@ -8417,10 +7642,10 @@
         </is>
       </c>
       <c r="AC62" t="n">
-        <v>4.090555556</v>
+        <v>4.1258314</v>
       </c>
       <c r="AD62" t="n">
-        <v>-76.22221999999999</v>
+        <v>-76.3722336</v>
       </c>
     </row>
     <row r="63">
@@ -8439,48 +7664,48 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>jueves</t>
+          <t>viernes</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>BID (43)</t>
+          <t>Tuluá</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>ALFREDO GARRIDO TOVAR</t>
+          <t>SEDE INSTITUTO CAMPESTRE SANTA CECILIA</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA ALFREDO GARRIDO TOVAR</t>
+          <t>INSTITUCION EDUCATIVA MODERNA DE TULUA</t>
         </is>
       </c>
       <c r="J63" s="3" t="inlineStr">
         <is>
-          <t>276616000654</t>
+          <t>176834000599</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>RIOFRIO</t>
+          <t>Tuluá</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>CORREG PORTUGAL DE PIEDRAS</t>
+          <t>IND CALLE 27 NO 6AW 240</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -8494,10 +7719,10 @@
         </is>
       </c>
       <c r="P63" t="n">
+        <v>9.890000000000001</v>
+      </c>
+      <c r="Q63" t="n">
         <v>32.44</v>
-      </c>
-      <c r="Q63" t="n">
-        <v>41.58</v>
       </c>
       <c r="R63" t="n">
         <v>84.09999999999999</v>
@@ -8505,29 +7730,19 @@
       <c r="S63" t="n">
         <v>59</v>
       </c>
-      <c r="T63" t="inlineStr">
-        <is>
-          <t>No habitable</t>
-        </is>
-      </c>
-      <c r="U63" t="inlineStr">
-        <is>
-          <t>aprobado por la mesa</t>
-        </is>
-      </c>
       <c r="V63" t="inlineStr">
         <is>
-          <t>Colapso parcial</t>
+          <t>Afectación parcial</t>
         </is>
       </c>
       <c r="W63" t="inlineStr">
         <is>
-          <t>Critico</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="X63" t="inlineStr">
         <is>
-          <t>camino rural sin categoria</t>
+          <t>camino destapado</t>
         </is>
       </c>
       <c r="Y63" t="inlineStr">
@@ -8537,12 +7752,7 @@
       </c>
       <c r="Z63" t="inlineStr">
         <is>
-          <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 36 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AA63" t="inlineStr">
-        <is>
-          <t>PORTUGAL DE PIEDRAS - CRUCE VIA 23VL13</t>
+          <t>OpenStreetMap la marca como «track», la clase de los caminos de uso agrícola o forestal. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 50 m de esa vía.</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
@@ -8551,10 +7761,10 @@
         </is>
       </c>
       <c r="AC63" t="n">
-        <v>4.0553</v>
+        <v>4.090555556</v>
       </c>
       <c r="AD63" t="n">
-        <v>-76.35465000000001</v>
+        <v>-76.22221999999999</v>
       </c>
     </row>
     <row r="64">
@@ -8580,7 +7790,7 @@
         <v>11</v>
       </c>
       <c r="F64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -8589,32 +7799,32 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>INTEGRADA DE TRUJILLO</t>
+          <t>ALFREDO GARRIDO TOVAR</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA INTEGRADA DE TRUJILLO</t>
+          <t>INSTITUCION EDUCATIVA ALFREDO GARRIDO TOVAR</t>
         </is>
       </c>
       <c r="J64" s="3" t="inlineStr">
         <is>
-          <t>176828000021</t>
+          <t>276616000654</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>TRUJILLO</t>
+          <t>RIOFRIO</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>Urbana</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>KR 18 15 40</t>
+          <t>CORREG PORTUGAL DE PIEDRAS</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -8628,16 +7838,16 @@
         </is>
       </c>
       <c r="P64" t="n">
-        <v>46.98</v>
+        <v>32.44</v>
       </c>
       <c r="Q64" t="n">
-        <v>0.67</v>
+        <v>41.58</v>
       </c>
       <c r="R64" t="n">
-        <v>91.90000000000001</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="S64" t="n">
-        <v>48.5</v>
+        <v>59</v>
       </c>
       <c r="T64" t="inlineStr">
         <is>
@@ -8651,32 +7861,32 @@
       </c>
       <c r="V64" t="inlineStr">
         <is>
-          <t>Afectación parcial</t>
+          <t>Colapso parcial</t>
         </is>
       </c>
       <c r="W64" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Critico</t>
         </is>
       </c>
       <c r="X64" t="inlineStr">
         <is>
-          <t>calle de casco urbano</t>
+          <t>camino rural sin categoria</t>
         </is>
       </c>
       <c r="Y64" t="inlineStr">
         <is>
-          <t>fácil</t>
+          <t>difícil</t>
         </is>
       </c>
       <c r="Z64" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 33 m de esa vía.</t>
+          <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 36 m de esa vía.</t>
         </is>
       </c>
       <c r="AA64" t="inlineStr">
         <is>
-          <t>Carrera 18</t>
+          <t>PORTUGAL DE PIEDRAS - CRUCE VIA 23VL13</t>
         </is>
       </c>
       <c r="AB64" t="inlineStr">
@@ -8685,10 +7895,10 @@
         </is>
       </c>
       <c r="AC64" t="n">
-        <v>4.208406</v>
+        <v>4.0553</v>
       </c>
       <c r="AD64" t="n">
-        <v>-76.31959500000001</v>
+        <v>-76.35465000000001</v>
       </c>
     </row>
     <row r="65">
@@ -8707,14 +7917,14 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>viernes</t>
+          <t>sábado</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -8723,7 +7933,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>SAGRADO CORAZON DE JESUS</t>
+          <t>INTEGRADA DE TRUJILLO</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -8733,7 +7943,7 @@
       </c>
       <c r="J65" s="3" t="inlineStr">
         <is>
-          <t>176828000064</t>
+          <t>176828000021</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -8748,7 +7958,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>KR 18 15 27</t>
+          <t>KR 18 15 40</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -8762,10 +7972,10 @@
         </is>
       </c>
       <c r="P65" t="n">
+        <v>46.98</v>
+      </c>
+      <c r="Q65" t="n">
         <v>0.67</v>
-      </c>
-      <c r="Q65" t="n">
-        <v>44.3</v>
       </c>
       <c r="R65" t="n">
         <v>91.90000000000001</v>
@@ -8773,14 +7983,24 @@
       <c r="S65" t="n">
         <v>48.5</v>
       </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>No habitable</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>aprobado por la mesa</t>
+        </is>
+      </c>
       <c r="V65" t="inlineStr">
         <is>
-          <t>Colapso parcial</t>
+          <t>Afectación parcial</t>
         </is>
       </c>
       <c r="W65" t="inlineStr">
         <is>
-          <t>Critico</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="X65" t="inlineStr">
@@ -8795,7 +8015,7 @@
       </c>
       <c r="Z65" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 26 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 33 m de esa vía.</t>
         </is>
       </c>
       <c r="AA65" t="inlineStr">
@@ -8809,10 +8029,10 @@
         </is>
       </c>
       <c r="AC65" t="n">
-        <v>4.210077</v>
+        <v>4.208406</v>
       </c>
       <c r="AD65" t="n">
-        <v>-76.319047</v>
+        <v>-76.31959500000001</v>
       </c>
     </row>
     <row r="66">
@@ -8838,7 +8058,7 @@
         <v>12</v>
       </c>
       <c r="F66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -8847,17 +8067,17 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>SAN ISIDRO</t>
+          <t>SAGRADO CORAZON DE JESUS</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA SAN ISIDRO</t>
+          <t>INSTITUCION EDUCATIVA INTEGRADA DE TRUJILLO</t>
         </is>
       </c>
       <c r="J66" s="3" t="inlineStr">
         <is>
-          <t>276828000174</t>
+          <t>176828000064</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -8867,12 +8087,12 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>CORREGIMIENTO EL TABOR PUENTE BLANCO</t>
+          <t>KR 18 15 27</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -8886,40 +8106,30 @@
         </is>
       </c>
       <c r="P66" t="n">
-        <v>77.20999999999999</v>
+        <v>0.67</v>
       </c>
       <c r="Q66" t="n">
-        <v>69.08</v>
+        <v>44.3</v>
       </c>
       <c r="R66" t="n">
-        <v>146.3</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="S66" t="n">
-        <v>74.2</v>
-      </c>
-      <c r="T66" t="inlineStr">
-        <is>
-          <t>Habitable</t>
-        </is>
-      </c>
-      <c r="U66" t="inlineStr">
-        <is>
-          <t>aprobado por la mesa</t>
-        </is>
+        <v>48.5</v>
       </c>
       <c r="V66" t="inlineStr">
         <is>
-          <t>Afectación parcial</t>
+          <t>Colapso parcial</t>
         </is>
       </c>
       <c r="W66" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Critico</t>
         </is>
       </c>
       <c r="X66" t="inlineStr">
         <is>
-          <t>via terciaria</t>
+          <t>calle de casco urbano</t>
         </is>
       </c>
       <c r="Y66" t="inlineStr">
@@ -8929,12 +8139,12 @@
       </c>
       <c r="Z66" t="inlineStr">
         <is>
-          <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 33 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 26 m de esa vía.</t>
         </is>
       </c>
       <c r="AA66" t="inlineStr">
         <is>
-          <t>TRUJILLO - LA SONORA CRUCE VIA 23VL13-1 K64+160</t>
+          <t>Carrera 18</t>
         </is>
       </c>
       <c r="AB66" t="inlineStr">
@@ -8943,10 +8153,10 @@
         </is>
       </c>
       <c r="AC66" t="n">
-        <v>4.210564</v>
+        <v>4.210077</v>
       </c>
       <c r="AD66" t="n">
-        <v>-76.38158300000001</v>
+        <v>-76.319047</v>
       </c>
     </row>
     <row r="67">
@@ -9658,7 +8868,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>

</xml_diff>